<commit_message>
Fix year-collision bug, update JIM001/FAM000 reconstructions to June 2026, and integrate Slice 005 Debtors Project OS
</commit_message>
<xml_diff>
--- a/analysis/debtors/FAM000/raw/FAM000_Final_Recon_Export.xlsx
+++ b/analysis/debtors/FAM000/raw/FAM000_Final_Recon_Export.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +487,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>41284.21</v>
+        <v>61626.77</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -498,88 +498,88 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46082</v>
+        <v>46083</v>
       </c>
       <c r="C3" t="n">
-        <v>20342.56</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>28807.5</v>
+        <v>-28807.5</v>
       </c>
       <c r="E3" t="n">
-        <v>49150.06</v>
+        <v>-28807.5</v>
       </c>
       <c r="F3" t="n">
         <v>61626.77</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>49501 / 49502</t>
+          <t>14518</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-28807.5</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>-28807.5</v>
+        <v>-18938.31</v>
       </c>
       <c r="F4" t="n">
-        <v>61626.77</v>
+        <v>42688.45999999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>14518</t>
+          <t>00043498</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46084</v>
+        <v>46088</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>11156.55</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>-18938.31</v>
+        <v>11156.55</v>
       </c>
       <c r="F5" t="n">
-        <v>42688.46</v>
+        <v>53845.00999999999</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>43498</t>
+          <t>49619</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -589,71 +589,71 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-27427.5</v>
+        <v>18975</v>
       </c>
       <c r="E6" t="n">
-        <v>-27427.5</v>
+        <v>18975</v>
       </c>
       <c r="F6" t="n">
-        <v>42688.46</v>
+        <v>53845.00999999999</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>14555</t>
+          <t>49620</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
         <v>46088</v>
       </c>
       <c r="C7" t="n">
-        <v>11156.55</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>18975</v>
+        <v>-27427.5</v>
       </c>
       <c r="E7" t="n">
-        <v>30131.55</v>
+        <v>-27427.5</v>
       </c>
       <c r="F7" t="n">
-        <v>53845.01</v>
+        <v>53845.00999999999</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>49619 / 49620</t>
+          <t>14555</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>46090</v>
       </c>
       <c r="C8" t="n">
-        <v>-863.74</v>
+        <v>863.74</v>
       </c>
       <c r="D8" t="n">
-        <v>-2070</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>-2933.74</v>
+        <v>863.74</v>
       </c>
       <c r="F8" t="n">
-        <v>52981.27</v>
+        <v>54708.74999999999</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>14559 / 14560</t>
+          <t>49626</t>
         </is>
       </c>
     </row>
@@ -667,263 +667,263 @@
         <v>46090</v>
       </c>
       <c r="C9" t="n">
-        <v>8925.17</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>10522.5</v>
+        <v>2070</v>
       </c>
       <c r="E9" t="n">
-        <v>19447.67</v>
+        <v>2070</v>
       </c>
       <c r="F9" t="n">
-        <v>61906.44</v>
+        <v>54708.74999999999</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>49626 / 49627 / 49628 / 49629</t>
+          <t>49627</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46091</v>
+        <v>46090</v>
       </c>
       <c r="C10" t="n">
+        <v>8061.43</v>
+      </c>
+      <c r="D10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="n">
-        <v>-20757.5</v>
-      </c>
       <c r="E10" t="n">
-        <v>-20757.5</v>
+        <v>8061.43</v>
       </c>
       <c r="F10" t="n">
-        <v>61906.44</v>
+        <v>62770.17999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>14571</t>
+          <t>49628</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>46091</v>
+        <v>46090</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>8452.5</v>
       </c>
       <c r="E11" t="n">
-        <v>-20343</v>
+        <v>8452.5</v>
       </c>
       <c r="F11" t="n">
-        <v>41563.44</v>
+        <v>62770.17999999999</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>43590 / 43590 / 43590 / 43590</t>
+          <t>49629</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46091</v>
+        <v>46090</v>
       </c>
       <c r="C12" t="n">
-        <v>13507.79</v>
+        <v>-863.74</v>
       </c>
       <c r="D12" t="n">
-        <v>20757.5</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>34265.29</v>
+        <v>-863.74</v>
       </c>
       <c r="F12" t="n">
-        <v>55071.23</v>
+        <v>61906.44</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>49668 / 49669</t>
+          <t>14559</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46093</v>
+        <v>46090</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>-2070</v>
       </c>
       <c r="E13" t="n">
-        <v>-11156.5</v>
+        <v>-2070</v>
       </c>
       <c r="F13" t="n">
-        <v>43914.73</v>
+        <v>61906.44</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>43612</t>
+          <t>14560</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>46095</v>
+        <v>46091</v>
       </c>
       <c r="C14" t="n">
-        <v>12955.92</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>12955.92</v>
+        <v>-20343</v>
       </c>
       <c r="F14" t="n">
-        <v>56870.65</v>
+        <v>41563.44</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>49746</t>
+          <t>00043590</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>46098</v>
+        <v>46091</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>13507.79</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>-12957</v>
+        <v>13507.79</v>
       </c>
       <c r="F15" t="n">
-        <v>43913.65</v>
+        <v>55071.23</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>43671 / 43671</t>
+          <t>49668</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>46100</v>
+        <v>46091</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>20757.5</v>
       </c>
       <c r="E16" t="n">
-        <v>-8062</v>
+        <v>20757.5</v>
       </c>
       <c r="F16" t="n">
-        <v>35851.65</v>
+        <v>55071.23</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>43702 / 43702</t>
+          <t>49669</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>46100</v>
+        <v>46091</v>
       </c>
       <c r="C17" t="n">
-        <v>16866.68</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>21390</v>
+        <v>-20757.5</v>
       </c>
       <c r="E17" t="n">
-        <v>38256.68</v>
+        <v>-20757.5</v>
       </c>
       <c r="F17" t="n">
-        <v>52718.33</v>
+        <v>55071.23</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>49832 / 49833</t>
+          <t>14571</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>46101</v>
+        <v>46093</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>-21390</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>-21390</v>
+        <v>-11156.5</v>
       </c>
       <c r="F18" t="n">
-        <v>52718.33</v>
+        <v>43914.73</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>14627</t>
+          <t>00043612</t>
         </is>
       </c>
     </row>
@@ -934,23 +934,23 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>46104</v>
+        <v>46095</v>
       </c>
       <c r="C19" t="n">
-        <v>18402.21</v>
+        <v>12955.92</v>
       </c>
       <c r="D19" t="n">
-        <v>24725</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>43127.21</v>
+        <v>12955.92</v>
       </c>
       <c r="F19" t="n">
-        <v>71120.53999999999</v>
+        <v>56870.64999999999</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>49871 / 49872</t>
+          <t>49746</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46105</v>
+        <v>46098</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -970,41 +970,41 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>-21600</v>
+        <v>-12957</v>
       </c>
       <c r="F20" t="n">
-        <v>49520.54</v>
+        <v>43913.64999999999</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>43741 / 43741</t>
+          <t>00043671</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>46106</v>
+        <v>46100</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>-24725</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>-24725</v>
+        <v>-8062</v>
       </c>
       <c r="F21" t="n">
-        <v>49520.54</v>
+        <v>35851.64999999999</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>14641</t>
+          <t>00043702</t>
         </is>
       </c>
     </row>
@@ -1015,131 +1015,131 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>46110</v>
+        <v>46100</v>
       </c>
       <c r="C22" t="n">
-        <v>25312.05</v>
+        <v>16866.68</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>25312.05</v>
+        <v>16866.68</v>
       </c>
       <c r="F22" t="n">
-        <v>74832.59</v>
+        <v>52718.32999999999</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>49991</t>
+          <t>49832</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>46111</v>
+        <v>46100</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>-34327.5</v>
+        <v>21390</v>
       </c>
       <c r="E23" t="n">
-        <v>-34327.5</v>
+        <v>21390</v>
       </c>
       <c r="F23" t="n">
-        <v>74832.59</v>
+        <v>52718.32999999999</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>14682</t>
+          <t>49833</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46111</v>
+        <v>46101</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>34845</v>
+        <v>-21390</v>
       </c>
       <c r="E24" t="n">
-        <v>34845</v>
+        <v>-21390</v>
       </c>
       <c r="F24" t="n">
-        <v>74832.59</v>
+        <v>52718.32999999999</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>49992</t>
+          <t>14627</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46112</v>
+        <v>46104</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>18402.21</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>-25312</v>
+        <v>18402.21</v>
       </c>
       <c r="F25" t="n">
-        <v>49520.59</v>
+        <v>71120.53999999999</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>43825 / 43826</t>
+          <t>49871</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>46119</v>
+        <v>46104</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>-53360</v>
+        <v>24725</v>
       </c>
       <c r="E26" t="n">
-        <v>-53360</v>
+        <v>24725</v>
       </c>
       <c r="F26" t="n">
-        <v>49520.59</v>
+        <v>71120.53999999999</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>14715 / 14716</t>
+          <t>49872</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46119</v>
+        <v>46105</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -1159,41 +1159,41 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>-37200</v>
+        <v>-21600</v>
       </c>
       <c r="F27" t="n">
-        <v>12320.59</v>
+        <v>49520.53999999999</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>43891 / 43891 / 43891 / 43892</t>
+          <t>00043741</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>46119</v>
+        <v>46106</v>
       </c>
       <c r="C28" t="n">
-        <v>40925.01</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>55372.5</v>
+        <v>-24725</v>
       </c>
       <c r="E28" t="n">
-        <v>96297.50999999999</v>
+        <v>-24725</v>
       </c>
       <c r="F28" t="n">
-        <v>53245.6</v>
+        <v>49520.53999999999</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>50102 / 50103 / 50111 / 50112</t>
+          <t>14641</t>
         </is>
       </c>
     </row>
@@ -1204,50 +1204,50 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>46122</v>
+        <v>46110</v>
       </c>
       <c r="C29" t="n">
-        <v>8920.83</v>
+        <v>25312.05</v>
       </c>
       <c r="D29" t="n">
-        <v>9890</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>18810.83</v>
+        <v>25312.05</v>
       </c>
       <c r="F29" t="n">
-        <v>62166.43</v>
+        <v>74832.59</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>50199 / 50200</t>
+          <t>49991</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>46124</v>
+        <v>46111</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>-12477.5</v>
+        <v>34845</v>
       </c>
       <c r="E30" t="n">
-        <v>-12477.5</v>
+        <v>34845</v>
       </c>
       <c r="F30" t="n">
-        <v>62166.43</v>
+        <v>74832.59</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>14743</t>
+          <t>49992</t>
         </is>
       </c>
     </row>
@@ -1258,23 +1258,23 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>46128</v>
+        <v>46111</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>-25587.5</v>
+        <v>-34327.5</v>
       </c>
       <c r="E31" t="n">
-        <v>-25587.5</v>
+        <v>-34327.5</v>
       </c>
       <c r="F31" t="n">
-        <v>62166.43</v>
+        <v>74832.59</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>14764</t>
+          <t>14682</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>46128</v>
+        <v>46112</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -1294,41 +1294,41 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>-21000</v>
+        <v>-25312</v>
       </c>
       <c r="F32" t="n">
-        <v>41166.43</v>
+        <v>49520.59</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>44007 / 44007 / 44007 / 44007 / 44007 / 44007 / 44007 / 44007 / 44007</t>
+          <t>00043825 / 00043826</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>46128</v>
+        <v>46119</v>
       </c>
       <c r="C33" t="n">
-        <v>20059.3</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>25587.5</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>45646.8</v>
+        <v>-37200</v>
       </c>
       <c r="F33" t="n">
-        <v>61225.73</v>
+        <v>12320.59</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>50254 / 50255</t>
+          <t>00043891 / 00043892</t>
         </is>
       </c>
     </row>
@@ -1339,77 +1339,77 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>46132</v>
+        <v>46119</v>
       </c>
       <c r="C34" t="n">
-        <v>12096.05</v>
+        <v>17463.68</v>
       </c>
       <c r="D34" t="n">
-        <v>12075</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>24171.05</v>
+        <v>17463.68</v>
       </c>
       <c r="F34" t="n">
-        <v>73321.78</v>
+        <v>29784.27</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>50316 / 50317</t>
+          <t>50102</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>46133</v>
+        <v>46119</v>
       </c>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>-14145</v>
+        <v>21965</v>
       </c>
       <c r="E35" t="n">
-        <v>-14145</v>
+        <v>21965</v>
       </c>
       <c r="F35" t="n">
-        <v>73321.78</v>
+        <v>29784.27</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>14782 / 14785</t>
+          <t>50103</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>46133</v>
+        <v>46119</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>23461.33</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>-16457.61</v>
+        <v>23461.33</v>
       </c>
       <c r="F36" t="n">
-        <v>56864.17</v>
+        <v>53245.6</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>44045 / 44046 / 44046 / 44046</t>
+          <t>50111</t>
         </is>
       </c>
     </row>
@@ -1420,23 +1420,23 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>46133</v>
+        <v>46119</v>
       </c>
       <c r="C37" t="n">
-        <v>2394.02</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>2070</v>
+        <v>33407.5</v>
       </c>
       <c r="E37" t="n">
-        <v>4464.02</v>
+        <v>33407.5</v>
       </c>
       <c r="F37" t="n">
-        <v>59258.19</v>
+        <v>53245.6</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>50322 / 50323 / 50324</t>
+          <t>50112</t>
         </is>
       </c>
     </row>
@@ -1447,158 +1447,158 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>46136</v>
+        <v>46119</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>-17422.5</v>
+        <v>-31222.5</v>
       </c>
       <c r="E38" t="n">
-        <v>-17422.5</v>
+        <v>-31222.5</v>
       </c>
       <c r="F38" t="n">
-        <v>59258.19</v>
+        <v>53245.6</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>14804</t>
+          <t>14715</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>46136</v>
+        <v>46119</v>
       </c>
       <c r="C39" t="n">
-        <v>13078.88</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>17422.5</v>
+        <v>-22137.5</v>
       </c>
       <c r="E39" t="n">
-        <v>30501.38</v>
+        <v>-22137.5</v>
       </c>
       <c r="F39" t="n">
-        <v>72337.07000000001</v>
+        <v>53245.6</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>50368 / 50369</t>
+          <t>14716</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>46140</v>
+        <v>46122</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>8920.83</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>-30000</v>
+        <v>8920.83</v>
       </c>
       <c r="F40" t="n">
-        <v>42337.07</v>
+        <v>62166.43</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>44102 / 44102 / 44102</t>
+          <t>50199</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>46141</v>
+        <v>46122</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>-20355</v>
+        <v>9890</v>
       </c>
       <c r="E41" t="n">
-        <v>-20355</v>
+        <v>9890</v>
       </c>
       <c r="F41" t="n">
-        <v>42337.07</v>
+        <v>62166.43</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>14813</t>
+          <t>50200</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>46141</v>
+        <v>46124</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>-12477.5</v>
       </c>
       <c r="E42" t="n">
-        <v>-30000</v>
+        <v>-12477.5</v>
       </c>
       <c r="F42" t="n">
-        <v>12337.07</v>
+        <v>62166.43</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>44102 / 44102 / 44102</t>
+          <t>14743</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>46141</v>
+        <v>46128</v>
       </c>
       <c r="C43" t="n">
-        <v>16254.09</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>20355</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>36609.09</v>
+        <v>-21000</v>
       </c>
       <c r="F43" t="n">
-        <v>28591.16</v>
+        <v>41166.43</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>50401 / 50402</t>
+          <t>00044007</t>
         </is>
       </c>
     </row>
@@ -1609,50 +1609,50 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>46143</v>
+        <v>46128</v>
       </c>
       <c r="C44" t="n">
-        <v>13078.88</v>
+        <v>20059.3</v>
       </c>
       <c r="D44" t="n">
-        <v>17422.5</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>30501.38</v>
+        <v>20059.3</v>
       </c>
       <c r="F44" t="n">
-        <v>41670.04</v>
+        <v>61225.73</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>50481 / 50482</t>
+          <t>50254</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>46145</v>
+        <v>46128</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>-17422.5</v>
+        <v>25587.5</v>
       </c>
       <c r="E45" t="n">
-        <v>-17422.5</v>
+        <v>25587.5</v>
       </c>
       <c r="F45" t="n">
-        <v>41670.04</v>
+        <v>61225.73</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>14839</t>
+          <t>50255</t>
         </is>
       </c>
     </row>
@@ -1663,23 +1663,23 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>46147</v>
+        <v>46128</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>-12995</v>
+        <v>-25587.5</v>
       </c>
       <c r="E46" t="n">
-        <v>-12995</v>
+        <v>-25587.5</v>
       </c>
       <c r="F46" t="n">
-        <v>41670.04</v>
+        <v>61225.73</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>14845</t>
+          <t>14764</t>
         </is>
       </c>
     </row>
@@ -1690,50 +1690,50 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46147</v>
+        <v>46132</v>
       </c>
       <c r="C47" t="n">
-        <v>13104.07</v>
+        <v>12096.05</v>
       </c>
       <c r="D47" t="n">
-        <v>12995</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>26099.07</v>
+        <v>12096.05</v>
       </c>
       <c r="F47" t="n">
-        <v>54774.11</v>
+        <v>73321.78</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>50498 / 50499</t>
+          <t>50316</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>46148</v>
+        <v>46132</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>-25300</v>
+        <v>12075</v>
       </c>
       <c r="E48" t="n">
-        <v>-25300</v>
+        <v>12075</v>
       </c>
       <c r="F48" t="n">
-        <v>54774.11</v>
+        <v>73321.78</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>14859</t>
+          <t>50317</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>46148</v>
+        <v>46133</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
@@ -1753,14 +1753,14 @@
         <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>-39000</v>
+        <v>-16457.61</v>
       </c>
       <c r="F49" t="n">
-        <v>15774.11</v>
+        <v>56864.17</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>44170 / 44170 / 44170</t>
+          <t>00044045 / 00044046</t>
         </is>
       </c>
     </row>
@@ -1771,50 +1771,50 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>46148</v>
+        <v>46133</v>
       </c>
       <c r="C50" t="n">
-        <v>17942.48</v>
+        <v>1436.41</v>
       </c>
       <c r="D50" t="n">
-        <v>25242.5</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>43184.98</v>
+        <v>1436.41</v>
       </c>
       <c r="F50" t="n">
-        <v>33716.59</v>
+        <v>58300.58</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>50526 / 50527</t>
+          <t>50322</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>46151</v>
+        <v>46133</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>2070</v>
       </c>
       <c r="E51" t="n">
-        <v>-10000</v>
+        <v>2070</v>
       </c>
       <c r="F51" t="n">
-        <v>23716.59</v>
+        <v>58300.58</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>44199 / 44199 / 44199</t>
+          <t>50323</t>
         </is>
       </c>
     </row>
@@ -1825,23 +1825,23 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>46153</v>
+        <v>46133</v>
       </c>
       <c r="C52" t="n">
-        <v>9772.18</v>
+        <v>957.61</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>9772.18</v>
+        <v>957.61</v>
       </c>
       <c r="F52" t="n">
-        <v>33488.77</v>
+        <v>59258.19</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>50610</t>
+          <t>50324</t>
         </is>
       </c>
     </row>
@@ -1852,50 +1852,50 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46154</v>
+        <v>46133</v>
       </c>
       <c r="C53" t="n">
         <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>-11212.5</v>
+        <v>-2070</v>
       </c>
       <c r="E53" t="n">
-        <v>-11212.5</v>
+        <v>-2070</v>
       </c>
       <c r="F53" t="n">
-        <v>33488.77</v>
+        <v>59258.19</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>14889</t>
+          <t>14782</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>46154</v>
+        <v>46133</v>
       </c>
       <c r="C54" t="n">
         <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>-12075</v>
       </c>
       <c r="E54" t="n">
-        <v>-19000</v>
+        <v>-12075</v>
       </c>
       <c r="F54" t="n">
-        <v>14488.77</v>
+        <v>59258.19</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>44245 / 44245</t>
+          <t>14785</t>
         </is>
       </c>
     </row>
@@ -1906,88 +1906,88 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>46154</v>
+        <v>46136</v>
       </c>
       <c r="C55" t="n">
+        <v>13078.88</v>
+      </c>
+      <c r="D55" t="n">
         <v>0</v>
       </c>
-      <c r="D55" t="n">
-        <v>11212.5</v>
-      </c>
       <c r="E55" t="n">
-        <v>11212.5</v>
+        <v>13078.88</v>
       </c>
       <c r="F55" t="n">
-        <v>14488.77</v>
+        <v>72337.07000000001</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>50611</t>
+          <t>50368</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>46155</v>
+        <v>46136</v>
       </c>
       <c r="C56" t="n">
         <v>0</v>
       </c>
       <c r="D56" t="n">
-        <v>-23115</v>
+        <v>17422.5</v>
       </c>
       <c r="E56" t="n">
-        <v>-23115</v>
+        <v>17422.5</v>
       </c>
       <c r="F56" t="n">
-        <v>14488.77</v>
+        <v>72337.07000000001</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>14901</t>
+          <t>50369</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>46155</v>
+        <v>46136</v>
       </c>
       <c r="C57" t="n">
-        <v>19807.51</v>
+        <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>23115</v>
+        <v>-17422.5</v>
       </c>
       <c r="E57" t="n">
-        <v>42922.51</v>
+        <v>-17422.5</v>
       </c>
       <c r="F57" t="n">
-        <v>34296.28</v>
+        <v>72337.07000000001</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>50650 / 50651</t>
+          <t>14804</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>46157</v>
+        <v>46140</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
@@ -1996,14 +1996,14 @@
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>0</v>
+        <v>-30000</v>
       </c>
       <c r="F58" t="n">
-        <v>34296.28</v>
+        <v>42337.07000000001</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>50714</t>
+          <t>00044102</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46158</v>
+        <v>46141</v>
       </c>
       <c r="C59" t="n">
         <v>0</v>
@@ -2023,14 +2023,14 @@
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>-14282.48</v>
+        <v>-30000</v>
       </c>
       <c r="F59" t="n">
-        <v>20013.8</v>
+        <v>12337.07000000001</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>44282 / 44282 / 44283 / 44292</t>
+          <t>00044102</t>
         </is>
       </c>
     </row>
@@ -2041,185 +2041,185 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>46158</v>
+        <v>46141</v>
       </c>
       <c r="C60" t="n">
-        <v>1282.48</v>
+        <v>16254.09</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>1282.48</v>
+        <v>16254.09</v>
       </c>
       <c r="F60" t="n">
-        <v>21296.28</v>
+        <v>28591.16000000001</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>50717</t>
+          <t>50401</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>46160</v>
+        <v>46141</v>
       </c>
       <c r="C61" t="n">
         <v>0</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>20355</v>
       </c>
       <c r="E61" t="n">
-        <v>-11856</v>
+        <v>20355</v>
       </c>
       <c r="F61" t="n">
-        <v>9440.280000000001</v>
+        <v>28591.16000000001</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>44311 / 44311</t>
+          <t>50402</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>46160</v>
+        <v>46141</v>
       </c>
       <c r="C62" t="n">
-        <v>11855.99</v>
+        <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>13800</v>
+        <v>-20355</v>
       </c>
       <c r="E62" t="n">
-        <v>25655.99</v>
+        <v>-20355</v>
       </c>
       <c r="F62" t="n">
-        <v>21296.27</v>
+        <v>28591.16000000001</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>50724 / 50725</t>
+          <t>14813</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>46161</v>
+        <v>46143</v>
       </c>
       <c r="C63" t="n">
+        <v>13078.88</v>
+      </c>
+      <c r="D63" t="n">
         <v>0</v>
       </c>
-      <c r="D63" t="n">
-        <v>-13800</v>
-      </c>
       <c r="E63" t="n">
-        <v>-13800</v>
+        <v>13078.88</v>
       </c>
       <c r="F63" t="n">
-        <v>21296.27</v>
+        <v>41670.04000000001</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>14925</t>
+          <t>50481</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>46162</v>
+        <v>46143</v>
       </c>
       <c r="C64" t="n">
         <v>0</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>17422.5</v>
       </c>
       <c r="E64" t="n">
-        <v>-10000</v>
+        <v>17422.5</v>
       </c>
       <c r="F64" t="n">
-        <v>11296.27</v>
+        <v>41670.04000000001</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>44335</t>
+          <t>50482</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Crd Note</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46162</v>
+        <v>46145</v>
       </c>
       <c r="C65" t="n">
-        <v>24310.52</v>
+        <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>27312.5</v>
+        <v>-17422.5</v>
       </c>
       <c r="E65" t="n">
-        <v>51623.02</v>
+        <v>-17422.5</v>
       </c>
       <c r="F65" t="n">
-        <v>35606.79</v>
+        <v>41670.04000000001</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>50794 / 50795 / 50796 / 50797</t>
+          <t>14839</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Crd Note</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46163</v>
+        <v>46147</v>
       </c>
       <c r="C66" t="n">
-        <v>-2565.01</v>
+        <v>13104.07</v>
       </c>
       <c r="D66" t="n">
-        <v>-27312.5</v>
+        <v>0</v>
       </c>
       <c r="E66" t="n">
-        <v>-29877.51</v>
+        <v>13104.07</v>
       </c>
       <c r="F66" t="n">
-        <v>33041.78</v>
+        <v>54774.11000000001</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>14933 / 14934 / 14935</t>
+          <t>50498</t>
         </is>
       </c>
     </row>
@@ -2230,23 +2230,23 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46167</v>
+        <v>46147</v>
       </c>
       <c r="C67" t="n">
-        <v>12853.48</v>
+        <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>21102.5</v>
+        <v>12995</v>
       </c>
       <c r="E67" t="n">
-        <v>33955.98</v>
+        <v>12995</v>
       </c>
       <c r="F67" t="n">
-        <v>45895.26</v>
+        <v>54774.11000000001</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>50863 / 50865</t>
+          <t>50499</t>
         </is>
       </c>
     </row>
@@ -2257,23 +2257,23 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46168</v>
+        <v>46147</v>
       </c>
       <c r="C68" t="n">
         <v>0</v>
       </c>
       <c r="D68" t="n">
-        <v>-21102.5</v>
+        <v>-12995</v>
       </c>
       <c r="E68" t="n">
-        <v>-21102.5</v>
+        <v>-12995</v>
       </c>
       <c r="F68" t="n">
-        <v>45895.26</v>
+        <v>54774.11000000001</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>14969</t>
+          <t>14845</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>46168</v>
+        <v>46148</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
@@ -2293,14 +2293,1256 @@
         <v>0</v>
       </c>
       <c r="E69" t="n">
+        <v>-39000</v>
+      </c>
+      <c r="F69" t="n">
+        <v>15774.11000000001</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>00044170</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C70" t="n">
+        <v>17942.48</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>17942.48</v>
+      </c>
+      <c r="F70" t="n">
+        <v>33716.59000000001</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>50526</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>25242.5</v>
+      </c>
+      <c r="E71" t="n">
+        <v>25242.5</v>
+      </c>
+      <c r="F71" t="n">
+        <v>33716.59000000001</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>50527</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" t="n">
+        <v>-25300</v>
+      </c>
+      <c r="E72" t="n">
+        <v>-25300</v>
+      </c>
+      <c r="F72" t="n">
+        <v>33716.59000000001</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>14859</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F73" t="n">
+        <v>23716.59000000001</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>00044199</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C74" t="n">
+        <v>9772.18</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="n">
+        <v>9772.18</v>
+      </c>
+      <c r="F74" t="n">
+        <v>33488.77000000001</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>50610</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>-19000</v>
+      </c>
+      <c r="F75" t="n">
+        <v>14488.77000000001</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>00044245</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" t="n">
+        <v>11212.5</v>
+      </c>
+      <c r="E76" t="n">
+        <v>11212.5</v>
+      </c>
+      <c r="F76" t="n">
+        <v>14488.77000000001</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>50611</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" t="n">
+        <v>-11212.5</v>
+      </c>
+      <c r="E77" t="n">
+        <v>-11212.5</v>
+      </c>
+      <c r="F77" t="n">
+        <v>14488.77000000001</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>14889</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C78" t="n">
+        <v>19807.51</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>19807.51</v>
+      </c>
+      <c r="F78" t="n">
+        <v>34296.28000000001</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>50650</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="n">
+        <v>23115</v>
+      </c>
+      <c r="E79" t="n">
+        <v>23115</v>
+      </c>
+      <c r="F79" t="n">
+        <v>34296.28000000001</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>50651</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" t="n">
+        <v>-23115</v>
+      </c>
+      <c r="E80" t="n">
+        <v>-23115</v>
+      </c>
+      <c r="F80" t="n">
+        <v>34296.28000000001</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>14901</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>46157</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F81" t="n">
+        <v>35796.28000000001</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>50714</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>46158</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>-14282.48</v>
+      </c>
+      <c r="F82" t="n">
+        <v>21513.80000000001</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>00044282 / 00044283 / 00044292</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>46158</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1282.48</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1282.48</v>
+      </c>
+      <c r="F83" t="n">
+        <v>22796.28000000001</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>50717</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>-11856</v>
+      </c>
+      <c r="F84" t="n">
+        <v>10940.28000000001</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>00044311</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="C85" t="n">
+        <v>11855.99</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>11855.99</v>
+      </c>
+      <c r="F85" t="n">
+        <v>22796.27000000001</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>50724</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="n">
+        <v>13800</v>
+      </c>
+      <c r="E86" t="n">
+        <v>13800</v>
+      </c>
+      <c r="F86" t="n">
+        <v>22796.27000000001</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>50725</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>46161</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="n">
+        <v>-13800</v>
+      </c>
+      <c r="E87" t="n">
+        <v>-13800</v>
+      </c>
+      <c r="F87" t="n">
+        <v>22796.27000000001</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>14925</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="F88" t="n">
+        <v>12796.27000000001</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>00044335</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C89" t="n">
+        <v>2565.01</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2565.01</v>
+      </c>
+      <c r="F89" t="n">
+        <v>15361.28000000001</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>50794</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C90" t="n">
+        <v>21745.51</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>21745.51</v>
+      </c>
+      <c r="F90" t="n">
+        <v>37106.79000000001</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>50795</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>3047.5</v>
+      </c>
+      <c r="E91" t="n">
+        <v>3047.5</v>
+      </c>
+      <c r="F91" t="n">
+        <v>37106.79000000001</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>50796</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" t="n">
+        <v>24265</v>
+      </c>
+      <c r="E92" t="n">
+        <v>24265</v>
+      </c>
+      <c r="F92" t="n">
+        <v>37106.79000000001</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>50797</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" t="n">
+        <v>-24265</v>
+      </c>
+      <c r="E93" t="n">
+        <v>-24265</v>
+      </c>
+      <c r="F93" t="n">
+        <v>37106.79000000001</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>14933</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C94" t="n">
+        <v>-2565.01</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>-2565.01</v>
+      </c>
+      <c r="F94" t="n">
+        <v>34541.78000000001</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>14934</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>-3047.5</v>
+      </c>
+      <c r="E95" t="n">
+        <v>-3047.5</v>
+      </c>
+      <c r="F95" t="n">
+        <v>34541.78000000001</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>14935</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>46167</v>
+      </c>
+      <c r="C96" t="n">
+        <v>12853.48</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
+        <v>12853.48</v>
+      </c>
+      <c r="F96" t="n">
+        <v>47395.26000000001</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>50863</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>46167</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" t="n">
+        <v>21102.5</v>
+      </c>
+      <c r="E97" t="n">
+        <v>21102.5</v>
+      </c>
+      <c r="F97" t="n">
+        <v>47395.26000000001</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>50865</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>46168</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
         <v>-21855</v>
       </c>
-      <c r="F69" t="n">
-        <v>24040.26</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>44405 / 44405 / 44405 / 44406 / 44406 / 44406 / 44406 / 44409 / 44409</t>
+      <c r="F98" t="n">
+        <v>25540.26000000001</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>00044405 / 00044406 / 00044409</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>46168</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" t="n">
+        <v>-21102.5</v>
+      </c>
+      <c r="E99" t="n">
+        <v>-21102.5</v>
+      </c>
+      <c r="F99" t="n">
+        <v>25540.26000000001</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>14969</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="C100" t="n">
+        <v>14307.01</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>14307.01</v>
+      </c>
+      <c r="F100" t="n">
+        <v>39847.27000000001</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>50942</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
+        <v>-19807</v>
+      </c>
+      <c r="F101" t="n">
+        <v>20040.27000000001</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>00044469 / 00044470</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C102" t="n">
+        <v>11485.48</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>11485.48</v>
+      </c>
+      <c r="F102" t="n">
+        <v>31525.75000000001</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>50963</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" t="n">
+        <v>15065</v>
+      </c>
+      <c r="E103" t="n">
+        <v>15065</v>
+      </c>
+      <c r="F103" t="n">
+        <v>31525.75000000001</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>50964</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C104" t="n">
+        <v>6840.03</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>6840.03</v>
+      </c>
+      <c r="F104" t="n">
+        <v>38365.78000000001</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>50969</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C105" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" t="n">
+        <v>-15065</v>
+      </c>
+      <c r="E105" t="n">
+        <v>-15065</v>
+      </c>
+      <c r="F105" t="n">
+        <v>38365.78000000001</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>-6840</v>
+      </c>
+      <c r="F106" t="n">
+        <v>31525.78000000001</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>00044498</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="C107" t="n">
+        <v>6840.03</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
+        <v>6840.03</v>
+      </c>
+      <c r="F107" t="n">
+        <v>38365.81000000001</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>51014</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C108" t="n">
+        <v>14799.29</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" t="n">
+        <v>14799.29</v>
+      </c>
+      <c r="F108" t="n">
+        <v>53165.10000000001</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>51045</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>-17000</v>
+      </c>
+      <c r="F109" t="n">
+        <v>36165.10000000001</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>00044519</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="n">
+        <v>-18500</v>
+      </c>
+      <c r="F110" t="n">
+        <v>17665.10000000001</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>00044566</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C111" t="n">
+        <v>14912.69</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="n">
+        <v>14912.69</v>
+      </c>
+      <c r="F111" t="n">
+        <v>32577.79000000002</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>51082</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="n">
+        <v>16847.5</v>
+      </c>
+      <c r="E112" t="n">
+        <v>16847.5</v>
+      </c>
+      <c r="F112" t="n">
+        <v>32577.79000000002</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>51083</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Crd Note</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="n">
+        <v>-16847.5</v>
+      </c>
+      <c r="E113" t="n">
+        <v>-16847.5</v>
+      </c>
+      <c r="F113" t="n">
+        <v>32577.79000000002</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>15026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C114" t="n">
+        <v>6634.18</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" t="n">
+        <v>6634.18</v>
+      </c>
+      <c r="F114" t="n">
+        <v>39211.97000000002</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>51109</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="n">
+        <v>8797.5</v>
+      </c>
+      <c r="E115" t="n">
+        <v>8797.5</v>
+      </c>
+      <c r="F115" t="n">
+        <v>39211.97000000002</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>51110</t>
         </is>
       </c>
     </row>
@@ -2315,7 +3557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G342"/>
+  <dimension ref="A1:G346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12923,6 +14165,130 @@
         <v>-2</v>
       </c>
       <c r="G342" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>50964</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>2</v>
+      </c>
+      <c r="G343" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G344" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>51083</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>1</v>
+      </c>
+      <c r="G345" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>15026</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G346" t="n">
         <v>23</v>
       </c>
     </row>
@@ -12937,7 +14303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G556"/>
+  <dimension ref="A1:G558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30179,6 +31545,68 @@
         <v>-1</v>
       </c>
       <c r="G556" t="n">
+        <v>-83</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>51083</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>2</v>
+      </c>
+      <c r="G557" t="n">
+        <v>-81</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>15026</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G558" t="n">
         <v>-83</v>
       </c>
     </row>
@@ -30193,7 +31621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G807"/>
+  <dimension ref="A1:G812"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55217,6 +56645,161 @@
       </c>
       <c r="G807" t="n">
         <v>74</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>50964</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F808" t="n">
+        <v>15</v>
+      </c>
+      <c r="G808" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F809" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G809" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>51083</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F810" t="n">
+        <v>10</v>
+      </c>
+      <c r="G810" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>15026</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F811" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G811" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>51110</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F812" t="n">
+        <v>10</v>
+      </c>
+      <c r="G812" t="n">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -58257,7 +59840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G716"/>
+  <dimension ref="A1:G721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80462,6 +82045,161 @@
         <v>1</v>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>50964</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>S.1</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F717" t="n">
+        <v>5</v>
+      </c>
+      <c r="G717" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>S.1</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F718" t="n">
+        <v>-5</v>
+      </c>
+      <c r="G718" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>51083</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>S.1</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>8</v>
+      </c>
+      <c r="G719" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>15026</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>S.1</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>In (Returned)</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>-8</v>
+      </c>
+      <c r="G720" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>51110</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>FAM000</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>S.1</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Out (Delivered)</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>3</v>
+      </c>
+      <c r="G721" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>